<commit_message>
Analysis on early signs of high risk customers
</commit_message>
<xml_diff>
--- a/Cleaned Dataset.xlsx
+++ b/Cleaned Dataset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data Analyst Portfolio\AuroraBank\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FD070D8-1E66-42DE-9131-91B5327092BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546042AE-7C52-4A3A-AC79-E2B8698329E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -411,7 +411,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -420,9 +420,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1053,8 +1050,8 @@
     <col min="9" max="9" width="14.46484375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.86328125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.06640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.1328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.3984375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1142,7 +1139,7 @@
       <c r="M2" s="2">
         <v>0.42</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1186,7 +1183,7 @@
       <c r="M3" s="2">
         <v>0.36</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1230,7 +1227,7 @@
       <c r="M4" s="2">
         <v>0.88</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="N4" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1274,7 +1271,7 @@
       <c r="M5" s="2">
         <v>0</v>
       </c>
-      <c r="N5" s="4" t="s">
+      <c r="N5" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1318,7 +1315,7 @@
       <c r="M6" s="2">
         <v>0.51</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="N6" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1362,7 +1359,7 @@
       <c r="M7" s="2">
         <v>0.3</v>
       </c>
-      <c r="N7" s="4" t="s">
+      <c r="N7" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1406,7 +1403,7 @@
       <c r="M8" s="2">
         <v>0.67</v>
       </c>
-      <c r="N8" s="4" t="s">
+      <c r="N8" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1450,7 +1447,7 @@
       <c r="M9" s="2">
         <v>0.92</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="N9" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1494,7 +1491,7 @@
       <c r="M10" s="2">
         <v>0.44</v>
       </c>
-      <c r="N10" s="4" t="s">
+      <c r="N10" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1538,7 +1535,7 @@
       <c r="M11" s="2">
         <v>0.21</v>
       </c>
-      <c r="N11" s="4" t="s">
+      <c r="N11" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1582,7 +1579,7 @@
       <c r="M12" s="2">
         <v>0.97</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="N12" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1626,7 +1623,7 @@
       <c r="M13" s="2">
         <v>0.39</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="N13" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1670,7 +1667,7 @@
       <c r="M14" s="2">
         <v>0.28000000000000003</v>
       </c>
-      <c r="N14" s="4" t="s">
+      <c r="N14" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1714,7 +1711,7 @@
       <c r="M15" s="2">
         <v>0.76</v>
       </c>
-      <c r="N15" s="4" t="s">
+      <c r="N15" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1758,7 +1755,7 @@
       <c r="M16" s="2">
         <v>0.61</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="N16" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1802,7 +1799,7 @@
       <c r="M17" s="2">
         <v>0.33</v>
       </c>
-      <c r="N17" s="4" t="s">
+      <c r="N17" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1846,7 +1843,7 @@
       <c r="M18" s="2">
         <v>0.84</v>
       </c>
-      <c r="N18" s="4" t="s">
+      <c r="N18" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1890,7 +1887,7 @@
       <c r="M19" s="2">
         <v>0.47</v>
       </c>
-      <c r="N19" s="5" t="s">
+      <c r="N19" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1934,7 +1931,7 @@
       <c r="M20" s="2">
         <v>0.37</v>
       </c>
-      <c r="N20" s="4" t="s">
+      <c r="N20" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1978,7 +1975,7 @@
       <c r="M21" s="2">
         <v>0.9</v>
       </c>
-      <c r="N21" s="4" t="s">
+      <c r="N21" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2022,7 +2019,7 @@
       <c r="M22" s="2">
         <v>0.49</v>
       </c>
-      <c r="N22" s="4" t="s">
+      <c r="N22" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2066,7 +2063,7 @@
       <c r="M23" s="2">
         <v>0.28999999999999998</v>
       </c>
-      <c r="N23" s="4" t="s">
+      <c r="N23" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2110,7 +2107,7 @@
       <c r="M24" s="2">
         <v>0.79</v>
       </c>
-      <c r="N24" s="4" t="s">
+      <c r="N24" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2154,7 +2151,7 @@
       <c r="M25" s="2">
         <v>0.41</v>
       </c>
-      <c r="N25" s="4" t="s">
+      <c r="N25" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2198,7 +2195,7 @@
       <c r="M26" s="2">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N26" s="4" t="s">
+      <c r="N26" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2242,7 +2239,7 @@
       <c r="M27" s="2">
         <v>0.81</v>
       </c>
-      <c r="N27" s="4" t="s">
+      <c r="N27" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2286,7 +2283,7 @@
       <c r="M28" s="2">
         <v>0.46</v>
       </c>
-      <c r="N28" s="4" t="s">
+      <c r="N28" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2330,7 +2327,7 @@
       <c r="M29" s="2">
         <v>0.26</v>
       </c>
-      <c r="N29" s="4" t="s">
+      <c r="N29" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2374,7 +2371,7 @@
       <c r="M30" s="2">
         <v>0.78</v>
       </c>
-      <c r="N30" s="4" t="s">
+      <c r="N30" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2418,7 +2415,7 @@
       <c r="M31" s="2">
         <v>0.43</v>
       </c>
-      <c r="N31" s="5" t="s">
+      <c r="N31" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2462,7 +2459,7 @@
       <c r="M32" s="2">
         <v>0.39</v>
       </c>
-      <c r="N32" s="4" t="s">
+      <c r="N32" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2506,7 +2503,7 @@
       <c r="M33" s="2">
         <v>0.93</v>
       </c>
-      <c r="N33" s="4" t="s">
+      <c r="N33" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2550,7 +2547,7 @@
       <c r="M34" s="2">
         <v>0.34</v>
       </c>
-      <c r="N34" s="4" t="s">
+      <c r="N34" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2594,7 +2591,7 @@
       <c r="M35" s="2">
         <v>0.31</v>
       </c>
-      <c r="N35" s="4" t="s">
+      <c r="N35" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2638,7 +2635,7 @@
       <c r="M36" s="2">
         <v>0.82</v>
       </c>
-      <c r="N36" s="4" t="s">
+      <c r="N36" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -2682,7 +2679,7 @@
       <c r="M37" s="2">
         <v>0.52</v>
       </c>
-      <c r="N37" s="4" t="s">
+      <c r="N37" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2726,7 +2723,7 @@
       <c r="M38" s="2">
         <v>0.48</v>
       </c>
-      <c r="N38" s="4" t="s">
+      <c r="N38" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2770,7 +2767,7 @@
       <c r="M39" s="2">
         <v>0.96</v>
       </c>
-      <c r="N39" s="4" t="s">
+      <c r="N39" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -2814,7 +2811,7 @@
       <c r="M40" s="2">
         <v>0.38</v>
       </c>
-      <c r="N40" s="5" t="s">
+      <c r="N40" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -2858,7 +2855,7 @@
       <c r="M41" s="2">
         <v>0.27</v>
       </c>
-      <c r="N41" s="4" t="s">
+      <c r="N41" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2902,7 +2899,7 @@
       <c r="M42" s="2">
         <v>0.8</v>
       </c>
-      <c r="N42" s="4" t="s">
+      <c r="N42" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -2946,7 +2943,7 @@
       <c r="M43" s="2">
         <v>0.45</v>
       </c>
-      <c r="N43" s="4" t="s">
+      <c r="N43" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -2990,7 +2987,7 @@
       <c r="M44" s="2">
         <v>0.51</v>
       </c>
-      <c r="N44" s="4" t="s">
+      <c r="N44" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3034,7 +3031,7 @@
       <c r="M45" s="2">
         <v>0.95</v>
       </c>
-      <c r="N45" s="4" t="s">
+      <c r="N45" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -3078,7 +3075,7 @@
       <c r="M46" s="2">
         <v>0.4</v>
       </c>
-      <c r="N46" s="4" t="s">
+      <c r="N46" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3122,7 +3119,7 @@
       <c r="M47" s="2">
         <v>0.28000000000000003</v>
       </c>
-      <c r="N47" s="4" t="s">
+      <c r="N47" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3166,7 +3163,7 @@
       <c r="M48" s="2">
         <v>0.83</v>
       </c>
-      <c r="N48" s="4" t="s">
+      <c r="N48" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3210,7 +3207,7 @@
       <c r="M49" s="2">
         <v>0.5</v>
       </c>
-      <c r="N49" s="4" t="s">
+      <c r="N49" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3254,7 +3251,7 @@
       <c r="M50" s="2">
         <v>0.53</v>
       </c>
-      <c r="N50" s="4" t="s">
+      <c r="N50" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3298,7 +3295,7 @@
       <c r="M51" s="2">
         <v>0.94</v>
       </c>
-      <c r="N51" s="4" t="s">
+      <c r="N51" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -3342,7 +3339,7 @@
       <c r="M52" s="2">
         <v>0.42</v>
       </c>
-      <c r="N52" s="4" t="s">
+      <c r="N52" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3386,7 +3383,7 @@
       <c r="M53" s="2">
         <v>0.3</v>
       </c>
-      <c r="N53" s="4" t="s">
+      <c r="N53" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3430,7 +3427,7 @@
       <c r="M54" s="2">
         <v>0.82</v>
       </c>
-      <c r="N54" s="4" t="s">
+      <c r="N54" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3474,7 +3471,7 @@
       <c r="M55" s="2">
         <v>0.44</v>
       </c>
-      <c r="N55" s="5" t="s">
+      <c r="N55" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3518,7 +3515,7 @@
       <c r="M56" s="2">
         <v>0.56000000000000005</v>
       </c>
-      <c r="N56" s="4" t="s">
+      <c r="N56" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3562,7 +3559,7 @@
       <c r="M57" s="2">
         <v>0.96</v>
       </c>
-      <c r="N57" s="4" t="s">
+      <c r="N57" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -3606,7 +3603,7 @@
       <c r="M58" s="2">
         <v>0.39</v>
       </c>
-      <c r="N58" s="4" t="s">
+      <c r="N58" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3650,7 +3647,7 @@
       <c r="M59" s="2">
         <v>0.27</v>
       </c>
-      <c r="N59" s="4" t="s">
+      <c r="N59" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3694,7 +3691,7 @@
       <c r="M60" s="2">
         <v>0.84</v>
       </c>
-      <c r="N60" s="4" t="s">
+      <c r="N60" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -3738,7 +3735,7 @@
       <c r="M61" s="2">
         <v>0.49</v>
       </c>
-      <c r="N61" s="4" t="s">
+      <c r="N61" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3782,7 +3779,7 @@
       <c r="M62" s="2">
         <v>0.52</v>
       </c>
-      <c r="N62" s="4" t="s">
+      <c r="N62" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3826,7 +3823,7 @@
       <c r="M63" s="2">
         <v>0.97</v>
       </c>
-      <c r="N63" s="4" t="s">
+      <c r="N63" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -3870,7 +3867,7 @@
       <c r="M64" s="2">
         <v>0.41</v>
       </c>
-      <c r="N64" s="4" t="s">
+      <c r="N64" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3914,7 +3911,7 @@
       <c r="M65" s="2">
         <v>0.28999999999999998</v>
       </c>
-      <c r="N65" s="4" t="s">
+      <c r="N65" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3958,7 +3955,7 @@
       <c r="M66" s="2">
         <v>0.83</v>
       </c>
-      <c r="N66" s="4" t="s">
+      <c r="N66" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4002,7 +3999,7 @@
       <c r="M67" s="2">
         <v>0.47</v>
       </c>
-      <c r="N67" s="5" t="s">
+      <c r="N67" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4046,7 +4043,7 @@
       <c r="M68" s="2">
         <v>0.55000000000000004</v>
       </c>
-      <c r="N68" s="4" t="s">
+      <c r="N68" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4090,7 +4087,7 @@
       <c r="M69" s="2">
         <v>0.95</v>
       </c>
-      <c r="N69" s="4" t="s">
+      <c r="N69" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -4134,7 +4131,7 @@
       <c r="M70" s="2">
         <v>0.4</v>
       </c>
-      <c r="N70" s="4" t="s">
+      <c r="N70" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4178,7 +4175,7 @@
       <c r="M71" s="2">
         <v>0.28000000000000003</v>
       </c>
-      <c r="N71" s="4" t="s">
+      <c r="N71" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4222,7 +4219,7 @@
       <c r="M72" s="2">
         <v>0.81</v>
       </c>
-      <c r="N72" s="4" t="s">
+      <c r="N72" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -4266,7 +4263,7 @@
       <c r="M73" s="2">
         <v>0.48</v>
       </c>
-      <c r="N73" s="4" t="s">
+      <c r="N73" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4310,7 +4307,7 @@
       <c r="M74" s="2">
         <v>0.51</v>
       </c>
-      <c r="N74" s="4" t="s">
+      <c r="N74" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4354,7 +4351,7 @@
       <c r="M75" s="2">
         <v>0.96</v>
       </c>
-      <c r="N75" s="4" t="s">
+      <c r="N75" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -4398,7 +4395,7 @@
       <c r="M76" s="2">
         <v>0.43</v>
       </c>
-      <c r="N76" s="4" t="s">
+      <c r="N76" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4442,7 +4439,7 @@
       <c r="M77" s="2">
         <v>0.3</v>
       </c>
-      <c r="N77" s="4" t="s">
+      <c r="N77" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4486,7 +4483,7 @@
       <c r="M78" s="2">
         <v>0.84</v>
       </c>
-      <c r="N78" s="4" t="s">
+      <c r="N78" s="2" t="s">
         <v>26</v>
       </c>
     </row>
@@ -4530,7 +4527,7 @@
       <c r="M79" s="2">
         <v>0.46</v>
       </c>
-      <c r="N79" s="5" t="s">
+      <c r="N79" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -4574,7 +4571,7 @@
       <c r="M80" s="2">
         <v>0.56999999999999995</v>
       </c>
-      <c r="N80" s="4" t="s">
+      <c r="N80" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -4618,7 +4615,7 @@
       <c r="M81" s="2">
         <v>0.97</v>
       </c>
-      <c r="N81" s="4" t="s">
+      <c r="N81" s="2" t="s">
         <v>37</v>
       </c>
     </row>

</xml_diff>